<commit_message>
feat: Update locomo data structure and improve memory context formatting
- Updated JSON files for locomo results, including metrics and response durations.
- Changed memory context format to reflect conversation episodes.
- Fixed timestamp parsing in locomo ingestion script.
- Removed outdated top10 evaluation files to streamline data management.
</commit_message>
<xml_diff>
--- a/evaluation/nemori_results/nemori-default/nemori_locomo_results.xlsx
+++ b/evaluation/nemori_results/nemori-default/nemori_locomo_results.xlsx
@@ -540,73 +540,73 @@
         <v>24</v>
       </c>
       <c r="B2">
-        <v>0.745021645021645</v>
+        <v>0.7525974025974026</v>
       </c>
       <c r="C2">
-        <v>0.001861975166026532</v>
+        <v>0.0009183204950475038</v>
       </c>
       <c r="D2">
-        <v>0.4574787088430223</v>
+        <v>0.4649466649596156</v>
       </c>
       <c r="E2">
-        <v>0.5130333589412324</v>
+        <v>0.5194215833394733</v>
       </c>
       <c r="F2">
-        <v>0.2609046957796077</v>
+        <v>0.2642064074866582</v>
       </c>
       <c r="G2">
-        <v>0.4912352298903875</v>
+        <v>0.4991749886937291</v>
       </c>
       <c r="H2">
-        <v>0.3787242560797237</v>
+        <v>0.3870859337759753</v>
       </c>
       <c r="I2">
-        <v>0.2593088720660863</v>
+        <v>0.2648409873148418</v>
       </c>
       <c r="J2">
-        <v>0.1885910251108822</v>
+        <v>0.1930371048051992</v>
       </c>
       <c r="K2">
-        <v>0.1478078041527355</v>
+        <v>0.1534213862542812</v>
       </c>
       <c r="L2">
-        <v>0.4102775344365611</v>
+        <v>0.4140479595347844</v>
       </c>
       <c r="M2">
-        <v>0.4595226608875945</v>
+        <v>0.4608763168242007</v>
       </c>
       <c r="N2">
-        <v>0.750419335783302</v>
+        <v>0.7547912832204398</v>
       </c>
       <c r="O2">
-        <v>7835.28051948052</v>
+        <v>4432.091558441559</v>
       </c>
       <c r="P2">
-        <v>2516.519189500189</v>
+        <v>2260.71462724116</v>
       </c>
       <c r="Q2">
-        <v>2367.340445518494</v>
+        <v>2219.54345703125</v>
       </c>
       <c r="R2">
-        <v>3991.758441925048</v>
+        <v>3394.407260417938</v>
       </c>
       <c r="S2">
-        <v>0.5760186678403384</v>
+        <v>0.3997808927065366</v>
       </c>
       <c r="T2">
-        <v>0.3361701965332031</v>
+        <v>0.16021728515625</v>
       </c>
       <c r="U2">
-        <v>0.9214878082275388</v>
+        <v>0.722861289978025</v>
       </c>
       <c r="V2">
-        <v>2517.09520816803</v>
+        <v>2261.114408133866</v>
       </c>
       <c r="W2">
-        <v>2367.724776268005</v>
+        <v>2219.68138217926</v>
       </c>
       <c r="X2">
-        <v>3992.619132995605</v>
+        <v>3394.702458381653</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -614,73 +614,73 @@
         <v>25</v>
       </c>
       <c r="B3">
-        <v>0.7030114226375908</v>
+        <v>0.7476635514018691</v>
       </c>
       <c r="C3">
-        <v>0.002937099818012659</v>
+        <v>0.002543603055849614</v>
       </c>
       <c r="D3">
-        <v>0.5451976096317922</v>
+        <v>0.5476560336315552</v>
       </c>
       <c r="E3">
-        <v>0.5819836878248092</v>
+        <v>0.5776051743341463</v>
       </c>
       <c r="F3">
-        <v>0.2161625152279358</v>
+        <v>0.1868071699847401</v>
       </c>
       <c r="G3">
-        <v>0.5454732788844938</v>
+        <v>0.5421702734786846</v>
       </c>
       <c r="H3">
-        <v>0.471104775369148</v>
+        <v>0.4710045021446589</v>
       </c>
       <c r="I3">
-        <v>0.2975221578573395</v>
+        <v>0.2906508601282294</v>
       </c>
       <c r="J3">
-        <v>0.1988002621719275</v>
+        <v>0.1956770118906513</v>
       </c>
       <c r="K3">
-        <v>0.1644567533118029</v>
+        <v>0.1683577170541026</v>
       </c>
       <c r="L3">
-        <v>0.4492878079829428</v>
+        <v>0.4401740394008266</v>
       </c>
       <c r="M3">
-        <v>0.5010516316553061</v>
+        <v>0.4845460795931956</v>
       </c>
       <c r="N3">
-        <v>0.7783359543556736</v>
+        <v>0.7799734421236865</v>
       </c>
       <c r="O3">
-        <v>7740.052959501558</v>
+        <v>4357.894080996884</v>
       </c>
       <c r="P3">
-        <v>2266.428172774033</v>
+        <v>2001.25644734344</v>
       </c>
       <c r="Q3">
-        <v>2091.833114624023</v>
+        <v>1835.071086883545</v>
       </c>
       <c r="R3">
-        <v>3999.443054199219</v>
+        <v>3459.506034851074</v>
       </c>
       <c r="S3">
-        <v>0.6662031571813091</v>
+        <v>0.4852456838542427</v>
       </c>
       <c r="T3">
-        <v>0.3006458282470703</v>
+        <v>0.1509189605712891</v>
       </c>
       <c r="U3">
-        <v>0.926971435546875</v>
+        <v>1.043796539306641</v>
       </c>
       <c r="V3">
-        <v>2267.094375931214</v>
+        <v>2001.741693027294</v>
       </c>
       <c r="W3">
-        <v>2092.070341110229</v>
+        <v>1835.186004638672</v>
       </c>
       <c r="X3">
-        <v>4000.358104705811</v>
+        <v>3459.671258926392</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -688,73 +688,73 @@
         <v>26</v>
       </c>
       <c r="B4">
-        <v>0.5555555555555556</v>
+        <v>0.5208333333333334</v>
       </c>
       <c r="C4">
-        <v>0.004910463758239896</v>
+        <v>0.008505172717997162</v>
       </c>
       <c r="D4">
-        <v>0.2889034573084994</v>
+        <v>0.271044716861234</v>
       </c>
       <c r="E4">
-        <v>0.2907524147248082</v>
+        <v>0.2822999452873931</v>
       </c>
       <c r="F4">
-        <v>0.07699639403724456</v>
+        <v>0.06216336160193831</v>
       </c>
       <c r="G4">
-        <v>0.2814283658117647</v>
+        <v>0.2788968668843148</v>
       </c>
       <c r="H4">
-        <v>0.2137468525947208</v>
+        <v>0.1988118361878818</v>
       </c>
       <c r="I4">
-        <v>0.1035496548158403</v>
+        <v>0.09368909030555654</v>
       </c>
       <c r="J4">
-        <v>0.07383173382763493</v>
+        <v>0.06843437000100801</v>
       </c>
       <c r="K4">
-        <v>0.05585451203553374</v>
+        <v>0.05401756159676263</v>
       </c>
       <c r="L4">
-        <v>0.2172655146174085</v>
+        <v>0.1954940344236118</v>
       </c>
       <c r="M4">
-        <v>0.2977152308897833</v>
+        <v>0.2762240479120616</v>
       </c>
       <c r="N4">
-        <v>0.6283456149200598</v>
+        <v>0.6236937151600918</v>
       </c>
       <c r="O4">
-        <v>7645.03125</v>
+        <v>4294.104166666667</v>
       </c>
       <c r="P4">
-        <v>2355.73885589838</v>
+        <v>2119.710013270378</v>
       </c>
       <c r="Q4">
-        <v>2152.966380119324</v>
+        <v>1924.981594085693</v>
       </c>
       <c r="R4">
-        <v>3555.765151977539</v>
+        <v>3427.249252796173</v>
       </c>
       <c r="S4">
-        <v>0.6539771954218546</v>
+        <v>0.3127579887708028</v>
       </c>
       <c r="T4">
-        <v>0.3660917282104492</v>
+        <v>0.1701116561889648</v>
       </c>
       <c r="U4">
-        <v>0.9165406227111816</v>
+        <v>0.4834532737731934</v>
       </c>
       <c r="V4">
-        <v>2356.392833093802</v>
+        <v>2120.022771259149</v>
       </c>
       <c r="W4">
-        <v>2153.454303741455</v>
+        <v>1925.188541412354</v>
       </c>
       <c r="X4">
-        <v>3556.127369403839</v>
+        <v>3427.373111248016</v>
       </c>
     </row>
     <row r="5" spans="1:24">
@@ -762,73 +762,73 @@
         <v>27</v>
       </c>
       <c r="B5">
-        <v>0.6501182033096927</v>
+        <v>0.6288416075650118</v>
       </c>
       <c r="C5">
-        <v>0.008845525737054208</v>
+        <v>0.003343294473695265</v>
       </c>
       <c r="D5">
-        <v>0.3609880855633937</v>
+        <v>0.3448859645525123</v>
       </c>
       <c r="E5">
-        <v>0.4124071616077319</v>
+        <v>0.3898358822537057</v>
       </c>
       <c r="F5">
-        <v>0.1615351997225329</v>
+        <v>0.1460732480662511</v>
       </c>
       <c r="G5">
-        <v>0.373899504605486</v>
+        <v>0.3525123740659996</v>
       </c>
       <c r="H5">
-        <v>0.2619241468539862</v>
+        <v>0.2554640689730048</v>
       </c>
       <c r="I5">
-        <v>0.1663301834756319</v>
+        <v>0.1540852227490801</v>
       </c>
       <c r="J5">
-        <v>0.1139072445218275</v>
+        <v>0.100735433693329</v>
       </c>
       <c r="K5">
-        <v>0.0826019833516576</v>
+        <v>0.07492135398407232</v>
       </c>
       <c r="L5">
-        <v>0.295374537524608</v>
+        <v>0.2796653861391734</v>
       </c>
       <c r="M5">
-        <v>0.3409984716030948</v>
+        <v>0.3350001606330232</v>
       </c>
       <c r="N5">
-        <v>0.7045038388975968</v>
+        <v>0.6965836176635526</v>
       </c>
       <c r="O5">
-        <v>7911.421985815603</v>
+        <v>4482.269503546099</v>
       </c>
       <c r="P5">
-        <v>2378.864043147852</v>
+        <v>2040.371637817816</v>
       </c>
       <c r="Q5">
-        <v>2024.749636650085</v>
+        <v>1942.475914955139</v>
       </c>
       <c r="R5">
-        <v>4332.426476478575</v>
+        <v>3351.014196872711</v>
       </c>
       <c r="S5">
-        <v>0.6255537060135645</v>
+        <v>0.4073998606796806</v>
       </c>
       <c r="T5">
-        <v>0.3074407577514648</v>
+        <v>0.1463890075683594</v>
       </c>
       <c r="U5">
-        <v>0.9555220603942868</v>
+        <v>0.2949953079223628</v>
       </c>
       <c r="V5">
-        <v>2379.489596853865</v>
+        <v>2040.779037678495</v>
       </c>
       <c r="W5">
-        <v>2025.367736816406</v>
+        <v>1942.639470100403</v>
       </c>
       <c r="X5">
-        <v>4333.155775070189</v>
+        <v>3351.12714767456</v>
       </c>
     </row>
     <row r="6" spans="1:24">
@@ -836,73 +836,73 @@
         <v>28</v>
       </c>
       <c r="B6">
-        <v>0.8145065398335315</v>
+        <v>0.8224336107808164</v>
       </c>
       <c r="C6">
-        <v>0.0009708639487844875</v>
+        <v>0.001121057124354402</v>
       </c>
       <c r="D6">
-        <v>0.4755950141450132</v>
+        <v>0.4957694915809653</v>
       </c>
       <c r="E6">
-        <v>0.5458306273374222</v>
+        <v>0.567733012887507</v>
       </c>
       <c r="F6">
-        <v>0.3322954625007118</v>
+        <v>0.3564238136693024</v>
       </c>
       <c r="G6">
-        <v>0.5338270488615906</v>
+        <v>0.5570870821571687</v>
       </c>
       <c r="H6">
-        <v>0.4014606589861601</v>
+        <v>0.4206814376957699</v>
       </c>
       <c r="I6">
-        <v>0.2936803468574532</v>
+        <v>0.3116646954567429</v>
       </c>
       <c r="J6">
-        <v>0.2228366291450198</v>
+        <v>0.2372030068507636</v>
       </c>
       <c r="K6">
-        <v>0.1738140405725866</v>
+        <v>0.1853895361717343</v>
       </c>
       <c r="L6">
-        <v>0.4559487606237442</v>
+        <v>0.4740843339357776</v>
       </c>
       <c r="M6">
-        <v>0.5018847715196795</v>
+        <v>0.5151280409771496</v>
       </c>
       <c r="N6">
-        <v>0.7690947374038832</v>
+        <v>0.779662216886187</v>
       </c>
       <c r="O6">
-        <v>7867.813317479191</v>
+        <v>4459.337693222355</v>
       </c>
       <c r="P6">
-        <v>2676.486941778702</v>
+        <v>2449.72680525037</v>
       </c>
       <c r="Q6">
-        <v>2526.470899581909</v>
+        <v>2424.813985824585</v>
       </c>
       <c r="R6">
-        <v>3940.585136413574</v>
+        <v>3373.960018157959</v>
       </c>
       <c r="S6">
-        <v>0.516087490086323</v>
+        <v>0.3745388616137783</v>
       </c>
       <c r="T6">
-        <v>0.3561973571777344</v>
+        <v>0.1680850982666016</v>
       </c>
       <c r="U6">
-        <v>0.9081363677978516</v>
+        <v>0.7202625274658203</v>
       </c>
       <c r="V6">
-        <v>2677.003029268789</v>
+        <v>2450.101344111984</v>
       </c>
       <c r="W6">
-        <v>2526.768922805786</v>
+        <v>2425.29296875</v>
       </c>
       <c r="X6">
-        <v>3940.861225128174</v>
+        <v>3374.157190322876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>